<commit_message>
Add ML step module, rules vs ML comparison table, and updated README
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="False Alarms" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missed" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ML vs Rules" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4456,4 +4457,84 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Approach</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Precision %</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Recall %</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Typo Duplicates Caught</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Detection Rules (Exact + Likely)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>81.0%</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0 / 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Logistic Regression ML Model</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>95.2%</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>3 / 4</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update ML step with StandardScaler, add MEMO.md, clean README, and add MIT LICENSE
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -4520,17 +4520,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>95.5%</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>95.2%</t>
-        </is>
-      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3 / 4</t>
+          <t>4 / 4</t>
         </is>
       </c>
     </row>

</xml_diff>